<commit_message>
docs(upload): refresh template guide/instructions — CSV now works on every page
Updates the downloadable guide and the .xlsx Instructions sheet to reflect that
.csv is now accepted on all three upload pages (Upload Data, Bank Statements,
Historical Data), removing the prior 'use .xlsx, CSV only on Historical Data'
caveat.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UNX4grovytj7zLjmyeanAS
</commit_message>
<xml_diff>
--- a/static/samples/Analee_Bank_Statement_Template.xlsx
+++ b/static/samples/Analee_Bank_Statement_Template.xlsx
@@ -728,14 +728,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 'Upload Data' and 'Bank Statements' pages: use the .xlsx file (CSV is not reliably read there).</t>
+          <t xml:space="preserve">  - Works on all three pages: Upload Data, Bank Statements, and Historical Data.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 'Historical Data' page: .xlsx or .csv both work.</t>
+          <t xml:space="preserve">  - Both .xlsx and .csv are accepted on every page.</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Max file size 40 MB. Allowed types: .xlsx (everywhere), .csv (Historical Data).</t>
+          <t xml:space="preserve">  - Max file size 40 MB. Allowed types: .xlsx and .csv (both work on every upload page).</t>
         </is>
       </c>
     </row>

</xml_diff>